<commit_message>
version of the meta and first runs
</commit_message>
<xml_diff>
--- a/code/resultados/NWJSSP_OADG_NEH(MS+ELS+PROBABILISTICO).xlsx
+++ b/code/resultados/NWJSSP_OADG_NEH(MS+ELS+PROBABILISTICO).xlsx
@@ -423,10 +423,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="B1" t="n">
-        <v>34</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="2">
@@ -434,16 +434,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="E2" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -465,10 +465,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>337</v>
+        <v>321</v>
       </c>
       <c r="B1" t="n">
-        <v>18</v>
+        <v>613</v>
       </c>
     </row>
     <row r="2">
@@ -476,19 +476,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E2" t="n">
         <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>67</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -507,42 +507,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>10316</v>
+        <v>9808</v>
       </c>
       <c r="B1" t="n">
-        <v>965</v>
+        <v>564343</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B2" t="n">
+        <v>201</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1135</v>
+      </c>
+      <c r="D2" t="n">
+        <v>979</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>755</v>
+      </c>
+      <c r="G2" t="n">
+        <v>552</v>
+      </c>
+      <c r="H2" t="n">
+        <v>604</v>
+      </c>
+      <c r="I2" t="n">
+        <v>84</v>
+      </c>
+      <c r="J2" t="n">
         <v>343</v>
-      </c>
-      <c r="B2" t="n">
-        <v>498</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1192</v>
-      </c>
-      <c r="D2" t="n">
-        <v>657</v>
-      </c>
-      <c r="E2" t="n">
-        <v>65</v>
-      </c>
-      <c r="F2" t="n">
-        <v>833</v>
-      </c>
-      <c r="G2" t="n">
-        <v>209</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1029</v>
-      </c>
-      <c r="I2" t="n">
-        <v>381</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -561,42 +561,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>10238</v>
+        <v>10077</v>
       </c>
       <c r="B1" t="n">
-        <v>400</v>
+        <v>402991</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>87</v>
+        <v>287</v>
       </c>
       <c r="B2" t="n">
-        <v>1039</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>791</v>
+        <v>1129</v>
       </c>
       <c r="D2" t="n">
-        <v>1112</v>
+        <v>929</v>
       </c>
       <c r="E2" t="n">
-        <v>416</v>
+        <v>560</v>
       </c>
       <c r="F2" t="n">
-        <v>228</v>
+        <v>166</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H2" t="n">
-        <v>622</v>
+        <v>766</v>
       </c>
       <c r="I2" t="n">
-        <v>483</v>
+        <v>627</v>
       </c>
       <c r="J2" t="n">
-        <v>351</v>
+        <v>495</v>
       </c>
     </row>
   </sheetData>
@@ -615,10 +615,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>17076</v>
+        <v>17527</v>
       </c>
       <c r="B1" t="n">
-        <v>9236</v>
+        <v>3600000</v>
       </c>
     </row>
     <row r="2">
@@ -626,13 +626,13 @@
         <v>167</v>
       </c>
       <c r="B2" t="n">
-        <v>1246</v>
+        <v>1188</v>
       </c>
       <c r="C2" t="n">
-        <v>554</v>
+        <v>887</v>
       </c>
       <c r="D2" t="n">
-        <v>1094</v>
+        <v>1034</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -647,10 +647,10 @@
         <v>119</v>
       </c>
       <c r="I2" t="n">
-        <v>1357</v>
+        <v>1299</v>
       </c>
       <c r="J2" t="n">
-        <v>835</v>
+        <v>480</v>
       </c>
       <c r="K2" t="n">
         <v>247</v>
@@ -659,25 +659,25 @@
         <v>254</v>
       </c>
       <c r="M2" t="n">
-        <v>1509</v>
+        <v>1022</v>
       </c>
       <c r="N2" t="n">
-        <v>981</v>
+        <v>1280</v>
       </c>
       <c r="O2" t="n">
-        <v>735</v>
+        <v>575</v>
       </c>
       <c r="P2" t="n">
-        <v>383</v>
+        <v>392</v>
       </c>
       <c r="Q2" t="n">
-        <v>760</v>
+        <v>742</v>
       </c>
       <c r="R2" t="n">
-        <v>834</v>
+        <v>1507</v>
       </c>
       <c r="S2" t="n">
-        <v>480</v>
+        <v>813</v>
       </c>
       <c r="T2" t="n">
         <v>23</v>
@@ -699,10 +699,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>18402</v>
+        <v>18478</v>
       </c>
       <c r="B1" t="n">
-        <v>11803</v>
+        <v>3600001</v>
       </c>
       <c r="C1" t="inlineStr"/>
       <c r="D1" t="inlineStr"/>
@@ -728,61 +728,61 @@
         <v>7</v>
       </c>
       <c r="B2" t="n">
+        <v>62</v>
+      </c>
+      <c r="C2" t="n">
         <v>1014</v>
       </c>
-      <c r="C2" t="n">
-        <v>189</v>
-      </c>
       <c r="D2" t="n">
-        <v>627</v>
+        <v>898</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>1061</v>
+        <v>104</v>
       </c>
       <c r="G2" t="n">
-        <v>907</v>
+        <v>299</v>
       </c>
       <c r="H2" t="n">
-        <v>980</v>
+        <v>445</v>
       </c>
       <c r="I2" t="n">
-        <v>1303</v>
+        <v>588</v>
       </c>
       <c r="J2" t="n">
-        <v>62</v>
+        <v>1480</v>
       </c>
       <c r="K2" t="n">
-        <v>304</v>
+        <v>392</v>
       </c>
       <c r="L2" t="n">
-        <v>1540</v>
+        <v>611</v>
       </c>
       <c r="M2" t="n">
-        <v>615</v>
+        <v>406</v>
       </c>
       <c r="N2" t="n">
-        <v>1288</v>
+        <v>1234</v>
       </c>
       <c r="O2" t="n">
-        <v>515</v>
+        <v>1193</v>
       </c>
       <c r="P2" t="n">
-        <v>60</v>
+        <v>1197</v>
       </c>
       <c r="Q2" t="n">
-        <v>836</v>
+        <v>929</v>
       </c>
       <c r="R2" t="n">
-        <v>1159</v>
+        <v>1479</v>
       </c>
       <c r="S2" t="n">
-        <v>437</v>
+        <v>756</v>
       </c>
       <c r="T2" t="n">
-        <v>389</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>